<commit_message>
§13.14: sync preset_matrix xlsx (librav1e preview=7, balanced=6); add bench concurrency guard; fill _EQQUAL_TIER_OVERRIDE with matrix values (pending T4/L40 calibration); state doc updated
</commit_message>
<xml_diff>
--- a/Accessory/preset_matrix.xlsx
+++ b/Accessory/preset_matrix.xlsx
@@ -659,12 +659,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>**native（暂留，§13.10.1）**</t>
+          <t>6（显式 -speed 6，与 native 逐字节相同，零回归）</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
docs(matrix): preset_matrix 两版补齐丢失三列；v3 §13.10/§13.10.1 旧口径修正；q3_bench 文本证据入库
- preset_matrix.xlsx / preset_matrix_final_rebuilt.xlsx：补回「级别范围/默认值/速度·质量倾向」
  三列（自 d05c04a 版逐格移植并校验）；档值零改动；表头行恢复加粗
- v3 文档 §13.10 表：librav1e preview 6→7、balanced「native（暂留）」→ 显式 -speed 6
  （与 native 逐字节相同，已复核实测 md5 一致）；libvpx-vp9 balanced 补「已拍板=2」；
  §13.10.1 理由段与 §13.14 注意事项同步
- q3_bench 新增文本证据 226 个文件入库（json/txt/log/py/tsv/sh/time 等）；
  23 个 mp4/webm 媒体（19MB）按「证据文本入库、编码样本不入库」惯例剔除、维持未跟踪；
  510 个被既有 `logs/` 忽略规则挡下的原始计时日志（2.1MB）未入库（汇总 tsv 已入库）
- Accessory/probe/_duration_check.py：拉长片段差分校验脚本（选项 2）入库
</commit_message>
<xml_diff>
--- a/Accessory/preset_matrix.xlsx
+++ b/Accessory/preset_matrix.xlsx
@@ -420,8 +420,8 @@
   <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.4" customWidth="1" min="1" max="1"/>
-    <col width="9.6" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="78" customWidth="1" min="3" max="3"/>
     <col width="7.9" customWidth="1" min="4" max="4"/>
     <col width="25.3" customWidth="1" min="5" max="5"/>
@@ -438,7 +438,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>编码器</t>
+          <t>Codec / 编码器</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>**balanced**</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>**恒等值（待定，§13.4）**</t>
+          <t>**恒等值（待定，§13.4，已拍板=2）**</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">

</xml_diff>

<commit_message>
docs(quality-tier)+fix: R1 审核修正落实（两方案改写 / 矩阵同步 / 占位清理 / harness --preset-override）
- v3 主方案：§13.15 R1 决策记录；§4.1 权威 TIER_PROFILES（=§13.10R=xlsx）；§4.4 窗口接管含 balanced；§4.4.1 HDR×tier；§9 契约改写；§12.7 台账合并
- Part B：H3 时序（harness 主测先行）；阈值 3%/1.5×/1% 定稿；A/B 对 p5↔p6、svtav1 5↔3；libx264 进 CPU 环；M7 锚点扩展
- convert_crf.py：_EQQUAL_TIER_OVERRIDE 非 balanced 清空（H4：缺键=未标定回退 balanced+告警）
- calibrate_equal_quality.py：--preset-override（PRESET_AXIS + _lock_for 统一替换，自测 4 例）
- preset_matrix.xlsx：x265 test=ultrafast；vp9 2/1/0/0/0；aom balanced=6、8/8/7；量程/默认列修正
</commit_message>
<xml_diff>
--- a/Accessory/preset_matrix.xlsx
+++ b/Accessory/preset_matrix.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>veryfast</t>
+          <t>ultrafast</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -649,12 +649,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>-2,13</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0,8</t>
+          <t>-8,8</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -746,22 +746,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>**恒等值（待定，§13.4，已拍板=2）**</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -783,12 +783,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0,10</t>
+          <t>-1,10</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>native（0）</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>auto（4/5/6/8）</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -870,17 +870,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>6</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>**恒等值（待定，§13.4）**</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>p1,p7</t>
+          <t>p1~p7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>p1,p7</t>
+          <t>p1~p7</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>p1,p7</t>
+          <t>p1~p7</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">

</xml_diff>